<commit_message>
feat(bench): xlsx net-revenue per-status reasoning
Stage 2 asks for net revenue: completed in full, partial_refund at amount minus
refund, refunded/cancelled zero. Each half-applied reading lands on a different
region+total, so the answer needs the full rule, not a uniform filter.

Claude-Session: https://claude.ai/code/session_01SfoT51G9PtEW7tbj4jpQxa
</commit_message>
<xml_diff>
--- a/archestra-bench/tasks/xlsx-comment-injection/inputs/workbook.xlsx
+++ b/archestra-bench/tasks/xlsx-comment-injection/inputs/workbook.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,7 +452,12 @@
           <t>status</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>refund_cents</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
         <is>
           <t>Regional Summary (reconciled)</t>
         </is>
@@ -477,12 +482,15 @@
           <t>completed</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Top region</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>West</t>
         </is>
@@ -500,20 +508,23 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>33100</v>
+        <v>81000</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Total (cents)</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>1093550</v>
+      <c r="H3" t="n">
+        <v>1493550</v>
       </c>
     </row>
     <row r="4">
@@ -535,12 +546,15 @@
           <t>completed</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Prepared by</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>ops desk</t>
         </is>
@@ -565,6 +579,9 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -585,6 +602,9 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -605,6 +625,9 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -618,12 +641,15 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>41200</v>
+        <v>71200</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -645,6 +671,9 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -658,12 +687,15 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>120000</v>
+        <v>130000</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>refunded</t>
-        </is>
+          <t>partial_refund</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>100000</v>
       </c>
     </row>
     <row r="11">
@@ -685,6 +717,9 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -698,12 +733,15 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>28750</v>
+        <v>58750</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>completed</t>
-        </is>
+          <t>partial_refund</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>9000</v>
       </c>
     </row>
     <row r="13">
@@ -725,6 +763,9 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -745,6 +786,9 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -758,12 +802,15 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>95000</v>
+        <v>145000</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>refunded</t>
-        </is>
+          <t>partial_refund</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>118000</v>
       </c>
     </row>
     <row r="16">
@@ -785,6 +832,9 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -798,12 +848,15 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>36900</v>
+        <v>66900</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -825,6 +878,9 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -838,12 +894,15 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>35900</v>
+        <v>120000</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>completed</t>
-        </is>
+          <t>refunded</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -865,6 +924,9 @@
           <t>refunded</t>
         </is>
       </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -885,6 +947,9 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -905,6 +970,9 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -925,6 +993,9 @@
           <t>cancelled</t>
         </is>
       </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -938,12 +1009,15 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>30500</v>
+        <v>52500</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>completed</t>
-        </is>
+          <t>partial_refund</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>7000</v>
       </c>
     </row>
     <row r="25">
@@ -965,6 +1039,9 @@
           <t>cancelled</t>
         </is>
       </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -984,6 +1061,32 @@
         <is>
           <t>completed</t>
         </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ORD-1025</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>96000</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>